<commit_message>
Update project plan: assign system testing to both Charlie and Andy; add .xlsx to .gitignore
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -35,7 +35,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,8 +50,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0092D050"/>
-        <bgColor rgb="0092D050"/>
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,13 +73,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +454,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
@@ -511,12 +518,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-10-29</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -540,12 +547,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-10-04</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -569,12 +576,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-10-04</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -590,7 +597,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -610,12 +617,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-10-04</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -637,12 +644,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-10-04</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -654,9 +661,9 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -676,12 +683,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-10-11</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -703,12 +710,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-10-11</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -720,9 +727,9 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -742,12 +749,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-10-11</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -769,12 +776,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-10-11</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -786,9 +793,9 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -804,12 +811,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-10-18</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -817,13 +824,13 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Charlie Brown</t>
+          <t>Charlie Brown, Andy Mcarthy</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -839,12 +846,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025-11-23</t>
+          <t>2025-10-18</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -856,9 +863,9 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -874,12 +881,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -887,9 +894,9 @@
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -905,12 +912,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -932,12 +939,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -949,9 +956,9 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -967,12 +974,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -984,9 +991,9 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1006,12 +1013,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1019,9 +1026,9 @@
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1041,12 +1048,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-10-29</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1068,12 +1075,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-10-29</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1085,9 +1092,9 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Green</t>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1145,7 +1152,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-10-04</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1169,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-11-11</t>
+          <t>2025-10-06</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1186,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2025-10-11</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1203,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1220,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1237,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1254,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-10-22</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1271,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-10-29</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1288,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-10-29</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1308,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1343,11 +1350,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Low_Level_Design</t>
+          <t>Low_Level_Design, system_testing</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1380,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>

</xml_diff>